<commit_message>
ajuste na mapa celulas FT
ajuste na mapa celulas FT
</commit_message>
<xml_diff>
--- a/saida_relatorios/Eletrogóes_S_A/Supervisório_UHE_Rondon/FT_2026-05.xlsx
+++ b/saida_relatorios/Eletrogóes_S_A/Supervisório_UHE_Rondon/FT_2026-05.xlsx
@@ -11462,14 +11462,22 @@
           <t>CIDADE:</t>
         </is>
       </c>
-      <c r="O4" s="153" t="n"/>
+      <c r="O4" s="153" t="inlineStr">
+        <is>
+          <t>Pimenta Bueno</t>
+        </is>
+      </c>
       <c r="P4" s="152" t="n"/>
       <c r="Q4" s="17" t="inlineStr">
         <is>
           <t>ESTADO:</t>
         </is>
       </c>
-      <c r="R4" s="153" t="n"/>
+      <c r="R4" s="153" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
       <c r="S4" s="17" t="n"/>
       <c r="T4" s="14" t="n"/>
       <c r="U4" s="18" t="n"/>
@@ -12729,7 +12737,7 @@
       </c>
       <c r="O27" s="223" t="inlineStr">
         <is>
-          <t>Realizadas atividades iniciais de capacitação, preparação do ambiente de desenvolvimento e alinhamento técnico para o início da modernização do sistema supervisório da UHE Rondon.</t>
+          <t>Realizadas atividades iniciais de preparação do ambiente de desenvolvimento e alinhamento técnico para o início da modernização do sistema supervisório da UHE Rondon.</t>
         </is>
       </c>
       <c r="P27" s="151" t="n"/>
@@ -12847,7 +12855,7 @@
         <v>0.3333333333333333</v>
       </c>
       <c r="F29" s="53" t="n">
-        <v>0.4166666666666667</v>
+        <v>0.4583333333333333</v>
       </c>
       <c r="G29" s="54" t="n">
         <v>0.5</v>
@@ -12858,7 +12866,7 @@
       <c r="I29" s="56" t="n"/>
       <c r="J29" s="55" t="n"/>
       <c r="K29" s="218" t="n">
-        <v>0.2916666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="L29" s="219" t="n">
         <v>0</v>
@@ -12926,12 +12934,12 @@
         <v>0.5416666666666666</v>
       </c>
       <c r="H30" s="55" t="n">
-        <v>0.7083333333333334</v>
+        <v>0.75</v>
       </c>
       <c r="I30" s="56" t="n"/>
       <c r="J30" s="55" t="n"/>
       <c r="K30" s="218" t="n">
-        <v>0.2916666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="L30" s="219" t="n">
         <v>0</v>
@@ -12944,7 +12952,7 @@
       </c>
       <c r="O30" s="223" t="inlineStr">
         <is>
-          <t>Criação e ajuste da tela referente ao Mancal Guia da Turbina, contemplando a organização dos elementos gráficos, adequação do layout e preparação da interface para integração das variáveis de processo e sinalizações operacionais.</t>
+          <t>Realizadas atividades de desenvolvimento e aprimoramento da interface gráfica dos sistemas da unidade geradora da UHE Rondon.</t>
         </is>
       </c>
       <c r="P30" s="151" t="n"/>
@@ -13170,12 +13178,12 @@
         <v>0.5416666666666666</v>
       </c>
       <c r="H34" s="55" t="n">
-        <v>0.7083333333333334</v>
+        <v>0.75</v>
       </c>
       <c r="I34" s="56" t="n"/>
       <c r="J34" s="55" t="n"/>
       <c r="K34" s="218" t="n">
-        <v>0.2916666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="L34" s="219" t="n">
         <v>0</v>
@@ -13239,12 +13247,12 @@
         <v>0.5416666666666666</v>
       </c>
       <c r="H35" s="55" t="n">
-        <v>0.7083333333333334</v>
+        <v>0.75</v>
       </c>
       <c r="I35" s="56" t="n"/>
       <c r="J35" s="55" t="n"/>
       <c r="K35" s="218" t="n">
-        <v>0.2916666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="L35" s="219" t="n">
         <v>0</v>
@@ -13326,7 +13334,7 @@
       </c>
       <c r="O36" s="223" t="inlineStr">
         <is>
-          <t>Realizadas atividades de continuidade no desenvolvimento e adequação das interfaces gráficas dos sistemas operacionais da UHE Rondon, visando a padronização visual e preparação do supervisório para validação junto ao cliente.</t>
+          <t>Realizadas atividades de continuidade no desenvolvimento e adequação das interfaces gráficas dos sistemas operacionais da UHE Rondon.</t>
         </is>
       </c>
       <c r="P36" s="151" t="n"/>
@@ -13436,17 +13444,37 @@
       </c>
       <c r="C38" s="52" t="n"/>
       <c r="D38" s="64" t="n"/>
-      <c r="E38" s="52" t="n"/>
-      <c r="F38" s="53" t="n"/>
-      <c r="G38" s="54" t="n"/>
-      <c r="H38" s="55" t="n"/>
+      <c r="E38" s="52" t="n">
+        <v>0.4166666666666667</v>
+      </c>
+      <c r="F38" s="53" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G38" s="54" t="n">
+        <v>0.5416666666666666</v>
+      </c>
+      <c r="H38" s="55" t="n">
+        <v>0.7916666666666666</v>
+      </c>
       <c r="I38" s="56" t="n"/>
       <c r="J38" s="55" t="n"/>
-      <c r="K38" s="218" t="n"/>
-      <c r="L38" s="219" t="n"/>
-      <c r="M38" s="219" t="n"/>
-      <c r="N38" s="219" t="n"/>
-      <c r="O38" s="222" t="n"/>
+      <c r="K38" s="218" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L38" s="219" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" s="219" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" s="219" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" s="223" t="inlineStr">
+        <is>
+          <t>Realizadas atividades de desenvolvimento, padronização e aprimoramento das interfaces gráficas dos sistemas operacionais da UHE Rondon.</t>
+        </is>
+      </c>
       <c r="P38" s="151" t="n"/>
       <c r="Q38" s="151" t="n"/>
       <c r="R38" s="151" t="n"/>

</xml_diff>